<commit_message>
Scale sample dataset to 80 containers and optimize UI for large datasets
</commit_message>
<xml_diff>
--- a/COLDGUARD_Du_Lieu_Mau.xlsx
+++ b/COLDGUARD_Du_Lieu_Mau.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,10 +450,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4.2</v>
+        <v>5.7</v>
       </c>
       <c r="C2" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D2" t="n">
         <v>16</v>
@@ -471,13 +471,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>4.1</v>
       </c>
       <c r="C3" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="D3" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -492,13 +492,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
       <c r="C4" t="n">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D4" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -513,13 +513,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.5</v>
+        <v>4.2</v>
       </c>
       <c r="C5" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D5" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -534,17 +534,17 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9.4</v>
+        <v>4.7</v>
       </c>
       <c r="C6" t="n">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="D6" t="n">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bất thường</t>
+          <t>Bình thường</t>
         </is>
       </c>
     </row>
@@ -555,10 +555,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5.3</v>
+        <v>4.4</v>
       </c>
       <c r="C7" t="n">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D7" t="n">
         <v>14</v>
@@ -576,17 +576,17 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6.8</v>
+        <v>6.4</v>
       </c>
       <c r="C8" t="n">
         <v>87</v>
       </c>
       <c r="D8" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Bình thường</t>
+          <t>Bất thường</t>
         </is>
       </c>
     </row>
@@ -597,17 +597,17 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8.6</v>
+        <v>6.4</v>
       </c>
       <c r="C9" t="n">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="D9" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Bất thường</t>
+          <t>Bình thường</t>
         </is>
       </c>
     </row>
@@ -618,13 +618,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4.9</v>
+        <v>6.6</v>
       </c>
       <c r="C10" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D10" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -639,15 +639,1485 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6.2</v>
+        <v>4.8</v>
       </c>
       <c r="C11" t="n">
+        <v>78</v>
+      </c>
+      <c r="D11" t="n">
+        <v>20</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MG011</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="C12" t="n">
+        <v>80</v>
+      </c>
+      <c r="D12" t="n">
+        <v>15</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>MG012</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="C13" t="n">
+        <v>84</v>
+      </c>
+      <c r="D13" t="n">
+        <v>18</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>MG013</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="C14" t="n">
+        <v>94</v>
+      </c>
+      <c r="D14" t="n">
+        <v>69</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>MG014</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="C15" t="n">
+        <v>80</v>
+      </c>
+      <c r="D15" t="n">
+        <v>13</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MG015</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="C16" t="n">
+        <v>80</v>
+      </c>
+      <c r="D16" t="n">
+        <v>11</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MG016</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C17" t="n">
+        <v>83</v>
+      </c>
+      <c r="D17" t="n">
+        <v>9</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>MG017</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="C18" t="n">
+        <v>91</v>
+      </c>
+      <c r="D18" t="n">
+        <v>38</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Bất thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>MG018</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="C19" t="n">
+        <v>88</v>
+      </c>
+      <c r="D19" t="n">
+        <v>25</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>MG019</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="C20" t="n">
+        <v>82</v>
+      </c>
+      <c r="D20" t="n">
+        <v>12</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>MG020</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="C21" t="n">
+        <v>80</v>
+      </c>
+      <c r="D21" t="n">
+        <v>18</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>MG021</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="C22" t="n">
+        <v>87</v>
+      </c>
+      <c r="D22" t="n">
+        <v>26</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>MG022</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="C23" t="n">
+        <v>88</v>
+      </c>
+      <c r="D23" t="n">
+        <v>30</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>MG023</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="C24" t="n">
+        <v>78</v>
+      </c>
+      <c r="D24" t="n">
+        <v>8</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>MG024</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="C25" t="n">
+        <v>87</v>
+      </c>
+      <c r="D25" t="n">
+        <v>34</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MG025</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="C26" t="n">
+        <v>79</v>
+      </c>
+      <c r="D26" t="n">
+        <v>9</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MG026</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C27" t="n">
+        <v>84</v>
+      </c>
+      <c r="D27" t="n">
+        <v>19</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>MG027</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="C28" t="n">
+        <v>89</v>
+      </c>
+      <c r="D28" t="n">
+        <v>27</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>MG028</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="C29" t="n">
+        <v>84</v>
+      </c>
+      <c r="D29" t="n">
+        <v>12</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>MG029</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="C30" t="n">
+        <v>80</v>
+      </c>
+      <c r="D30" t="n">
+        <v>19</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>MG030</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="C31" t="n">
+        <v>93</v>
+      </c>
+      <c r="D31" t="n">
+        <v>52</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>MG031</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C32" t="n">
+        <v>84</v>
+      </c>
+      <c r="D32" t="n">
+        <v>12</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>MG032</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="C33" t="n">
+        <v>80</v>
+      </c>
+      <c r="D33" t="n">
+        <v>21</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>MG033</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>9</v>
+      </c>
+      <c r="C34" t="n">
+        <v>93</v>
+      </c>
+      <c r="D34" t="n">
+        <v>48</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>MG034</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>5</v>
+      </c>
+      <c r="C35" t="n">
+        <v>81</v>
+      </c>
+      <c r="D35" t="n">
+        <v>8</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>MG035</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="C36" t="n">
+        <v>79</v>
+      </c>
+      <c r="D36" t="n">
+        <v>10</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>MG036</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="C37" t="n">
+        <v>79</v>
+      </c>
+      <c r="D37" t="n">
+        <v>17</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>MG037</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="C38" t="n">
+        <v>88</v>
+      </c>
+      <c r="D38" t="n">
+        <v>29</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>MG038</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>7</v>
+      </c>
+      <c r="C39" t="n">
+        <v>85</v>
+      </c>
+      <c r="D39" t="n">
+        <v>34</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>MG039</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="C40" t="n">
+        <v>82</v>
+      </c>
+      <c r="D40" t="n">
+        <v>17</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>MG040</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="C41" t="n">
+        <v>79</v>
+      </c>
+      <c r="D41" t="n">
+        <v>17</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>MG041</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="C42" t="n">
+        <v>80</v>
+      </c>
+      <c r="D42" t="n">
+        <v>21</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>MG042</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C43" t="n">
+        <v>78</v>
+      </c>
+      <c r="D43" t="n">
+        <v>20</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>MG043</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>94</v>
+      </c>
+      <c r="D44" t="n">
+        <v>65</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Bất thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>MG044</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="C45" t="n">
+        <v>78</v>
+      </c>
+      <c r="D45" t="n">
+        <v>20</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>MG045</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="C46" t="n">
+        <v>92</v>
+      </c>
+      <c r="D46" t="n">
+        <v>49</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Bất thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>MG046</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>95</v>
+      </c>
+      <c r="D47" t="n">
+        <v>59</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>MG047</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="C48" t="n">
+        <v>82</v>
+      </c>
+      <c r="D48" t="n">
+        <v>8</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>MG048</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="C49" t="n">
+        <v>78</v>
+      </c>
+      <c r="D49" t="n">
+        <v>10</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>MG049</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="C50" t="n">
+        <v>82</v>
+      </c>
+      <c r="D50" t="n">
+        <v>11</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>MG050</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="C51" t="n">
         <v>86</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D51" t="n">
+        <v>33</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>MG051</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="C52" t="n">
+        <v>87</v>
+      </c>
+      <c r="D52" t="n">
+        <v>26</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>MG052</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="C53" t="n">
+        <v>84</v>
+      </c>
+      <c r="D53" t="n">
+        <v>13</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>MG053</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="C54" t="n">
+        <v>95</v>
+      </c>
+      <c r="D54" t="n">
+        <v>55</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Bất thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>MG054</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="C55" t="n">
+        <v>83</v>
+      </c>
+      <c r="D55" t="n">
+        <v>11</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>MG055</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="C56" t="n">
+        <v>79</v>
+      </c>
+      <c r="D56" t="n">
+        <v>21</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>MG056</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="C57" t="n">
+        <v>92</v>
+      </c>
+      <c r="D57" t="n">
+        <v>38</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Bất thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>MG057</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="C58" t="n">
+        <v>84</v>
+      </c>
+      <c r="D58" t="n">
+        <v>19</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>MG058</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="C59" t="n">
+        <v>83</v>
+      </c>
+      <c r="D59" t="n">
+        <v>12</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>MG059</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="C60" t="n">
+        <v>84</v>
+      </c>
+      <c r="D60" t="n">
+        <v>17</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>MG060</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>4</v>
+      </c>
+      <c r="C61" t="n">
+        <v>82</v>
+      </c>
+      <c r="D61" t="n">
+        <v>21</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>MG061</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="C62" t="n">
+        <v>84</v>
+      </c>
+      <c r="D62" t="n">
+        <v>18</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>MG062</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="C63" t="n">
+        <v>86</v>
+      </c>
+      <c r="D63" t="n">
         <v>28</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>MG063</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="C64" t="n">
+        <v>89</v>
+      </c>
+      <c r="D64" t="n">
+        <v>30</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>MG064</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="C65" t="n">
+        <v>88</v>
+      </c>
+      <c r="D65" t="n">
+        <v>33</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>MG065</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="C66" t="n">
+        <v>78</v>
+      </c>
+      <c r="D66" t="n">
+        <v>16</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>MG066</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="C67" t="n">
+        <v>81</v>
+      </c>
+      <c r="D67" t="n">
+        <v>12</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>MG067</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="C68" t="n">
+        <v>78</v>
+      </c>
+      <c r="D68" t="n">
+        <v>19</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>MG068</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C69" t="n">
+        <v>81</v>
+      </c>
+      <c r="D69" t="n">
+        <v>18</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>MG069</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>5</v>
+      </c>
+      <c r="C70" t="n">
+        <v>78</v>
+      </c>
+      <c r="D70" t="n">
+        <v>8</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>MG070</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="C71" t="n">
+        <v>82</v>
+      </c>
+      <c r="D71" t="n">
+        <v>18</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>MG071</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="C72" t="n">
+        <v>92</v>
+      </c>
+      <c r="D72" t="n">
+        <v>65</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>MG072</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>4</v>
+      </c>
+      <c r="C73" t="n">
+        <v>78</v>
+      </c>
+      <c r="D73" t="n">
+        <v>21</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>MG073</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="C74" t="n">
+        <v>87</v>
+      </c>
+      <c r="D74" t="n">
+        <v>26</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>MG074</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="C75" t="n">
+        <v>83</v>
+      </c>
+      <c r="D75" t="n">
+        <v>17</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>MG075</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="C76" t="n">
+        <v>83</v>
+      </c>
+      <c r="D76" t="n">
+        <v>15</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>MG076</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="C77" t="n">
+        <v>86</v>
+      </c>
+      <c r="D77" t="n">
+        <v>28</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>MG077</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>4</v>
+      </c>
+      <c r="C78" t="n">
+        <v>78</v>
+      </c>
+      <c r="D78" t="n">
+        <v>8</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>MG078</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="C79" t="n">
+        <v>93</v>
+      </c>
+      <c r="D79" t="n">
+        <v>41</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Bất thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>MG079</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C80" t="n">
+        <v>81</v>
+      </c>
+      <c r="D80" t="n">
+        <v>13</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>MG080</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="C81" t="n">
+        <v>85</v>
+      </c>
+      <c r="D81" t="n">
+        <v>29</v>
+      </c>
+      <c r="E81" t="inlineStr">
         <is>
           <t>Bình thường</t>
         </is>

</xml_diff>